<commit_message>
Add research activity to BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V75"/>
+  <dimension ref="A1:V76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4622,36 +4622,19 @@
           <t>plan</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
-      <c r="T69" t="inlineStr"/>
       <c r="U69" t="n">
         <v>0</v>
       </c>
-      <c r="V69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4828,80 +4811,66 @@
       <c r="V72" s="2" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050551</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>research study participants</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>A population that is studied in a research study.</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>human population</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="n"/>
-      <c r="F73" s="2" t="n"/>
-      <c r="G73" s="2" t="n"/>
-      <c r="H73" s="2" t="n"/>
-      <c r="I73" s="2" t="n"/>
-      <c r="J73" s="2" t="n"/>
-      <c r="K73" s="2" t="n"/>
-      <c r="L73" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M73" s="2" t="n"/>
-      <c r="N73" s="2" t="n"/>
-      <c r="O73" s="2" t="n"/>
-      <c r="P73" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Q73" s="2" t="n"/>
-      <c r="R73" s="2" t="n"/>
-      <c r="S73" s="2" t="n"/>
-      <c r="T73" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="U73" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V73" s="2" t="n"/>
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SEPIO:0000004</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>research activity</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
+      <c r="U73" t="n">
+        <v>0</v>
+      </c>
+      <c r="V73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010083</t>
+          <t>BCIO:050551</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>researcher role</t>
+          <t>research study participants</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>A occupational role played by a person that contributes substantively to production or reporting of a research study.</t>
+          <t>A population that is studied in a research study.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>occupational role of source</t>
+          <t>human population</t>
         </is>
       </c>
       <c r="E74" s="2" t="n"/>
@@ -4911,7 +4880,11 @@
       <c r="I74" s="2" t="n"/>
       <c r="J74" s="2" t="n"/>
       <c r="K74" s="2" t="n"/>
-      <c r="L74" s="2" t="n"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="M74" s="2" t="n"/>
       <c r="N74" s="2" t="n"/>
       <c r="O74" s="2" t="n"/>
@@ -4923,42 +4896,44 @@
       <c r="Q74" s="2" t="n"/>
       <c r="R74" s="2" t="n"/>
       <c r="S74" s="2" t="n"/>
-      <c r="T74" s="2" t="n"/>
-      <c r="U74" s="2" t="n">
-        <v>0</v>
+      <c r="T74" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U74" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="V74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>BCIO:051028</t>
+          <t>BCIO:010083</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>temporal context of process</t>
+          <t>researcher role</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>An occurrent that is not dependent on a process but may influence the effect of the process on its outcome.</t>
+          <t>A occupational role played by a person that contributes substantively to production or reporting of a research study.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>occurrent</t>
+          <t>occupational role of source</t>
         </is>
       </c>
       <c r="E75" s="2" t="n"/>
       <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="2" t="n"/>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This entity includes time periods, events, etc. </t>
-        </is>
-      </c>
+      <c r="I75" s="2" t="n"/>
       <c r="J75" s="2" t="n"/>
       <c r="K75" s="2" t="n"/>
       <c r="L75" s="2" t="n"/>
@@ -4979,6 +4954,56 @@
       </c>
       <c r="V75" s="2" t="n"/>
     </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:051028</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>temporal context of process</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>An occurrent that is not dependent on a process but may influence the effect of the process on its outcome.</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="n"/>
+      <c r="H76" s="2" t="n"/>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This entity includes time periods, events, etc. </t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="n"/>
+      <c r="K76" s="2" t="n"/>
+      <c r="L76" s="2" t="n"/>
+      <c r="M76" s="2" t="n"/>
+      <c r="N76" s="2" t="n"/>
+      <c r="O76" s="2" t="n"/>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q76" s="2" t="n"/>
+      <c r="R76" s="2" t="n"/>
+      <c r="S76" s="2" t="n"/>
+      <c r="T76" s="2" t="n"/>
+      <c r="U76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V76" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>